<commit_message>
Repeated analysis 18 nov with corrected counts. Included X-ray dose uncertainty
</commit_message>
<xml_diff>
--- a/Cell survival results/Analysis Results 18 November/Proton high.xlsx
+++ b/Cell survival results/Analysis Results 18 November/Proton high.xlsx
@@ -473,13 +473,13 @@
         <v>500</v>
       </c>
       <c r="D2" t="n">
-        <v>184</v>
+        <v>237</v>
       </c>
       <c r="E2" t="n">
-        <v>117</v>
+        <v>158</v>
       </c>
       <c r="F2" t="n">
-        <v>124</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3">
@@ -495,13 +495,13 @@
         <v>1000</v>
       </c>
       <c r="D3" t="n">
-        <v>131</v>
+        <v>53</v>
       </c>
       <c r="E3" t="n">
-        <v>94</v>
+        <v>32</v>
       </c>
       <c r="F3" t="n">
-        <v>87</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4">
@@ -514,16 +514,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>4000</v>
+        <v>8000</v>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="F4" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -536,16 +536,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>8000</v>
+        <v>16000</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>